<commit_message>
Fix some component model numbers
</commit_message>
<xml_diff>
--- a/ATX PSU Bench Supply.xlsx
+++ b/ATX PSU Bench Supply.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TNT_SAMUEL\Documents\KiCad\7.0\projects\ATX PSU Bench Supply\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352B74CC-6653-43C0-B91C-B6A457E8D417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA74E45-F7FA-428A-AF9F-0D3D7A0365F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A80751B4-A150-4C26-A609-D086283032E0}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="133">
   <si>
     <t>Source:</t>
   </si>
@@ -143,18 +143,9 @@
     <t>Connector:Conn_01x01_Socket</t>
   </si>
   <si>
-    <t>LIB_973582101:973582101</t>
-  </si>
-  <si>
-    <t>845-973582101</t>
-  </si>
-  <si>
     <t>J9</t>
   </si>
   <si>
-    <t>Molex 39-30-1241</t>
-  </si>
-  <si>
     <t>Connector:ATX-24</t>
   </si>
   <si>
@@ -164,30 +155,15 @@
     <t>https://www.intel.com/content/dam/www/public/us/en/documents/guides/power-supply-design-guide-june.pdf#page=33</t>
   </si>
   <si>
-    <t>39-30-1241</t>
-  </si>
-  <si>
-    <t>538-39-30-1241</t>
-  </si>
-  <si>
     <t>J10</t>
   </si>
   <si>
-    <t>Molex 46991-1008</t>
-  </si>
-  <si>
     <t>Connector_Generic:Conn_02x04_Top_Bottom</t>
   </si>
   <si>
     <t>Connector_Molex:Molex_Mini-Fit_Jr_5569-08A2_2x04_P4.20mm_Horizontal</t>
   </si>
   <si>
-    <t>46991-1008</t>
-  </si>
-  <si>
-    <t>538-46991-1008</t>
-  </si>
-  <si>
     <t>J11</t>
   </si>
   <si>
@@ -197,12 +173,6 @@
     <t>KLEEB_display:OLED-128x64</t>
   </si>
   <si>
-    <t>ADDR: 0x78/0x7A</t>
-  </si>
-  <si>
-    <t>J12, J13, J14, J15, J16, J17</t>
-  </si>
-  <si>
     <t>Conn_01x02</t>
   </si>
   <si>
@@ -290,9 +260,6 @@
     <t>504-MSMA2512R0050FEN</t>
   </si>
   <si>
-    <t>R16, R17, R19</t>
-  </si>
-  <si>
     <t>1.65k</t>
   </si>
   <si>
@@ -329,12 +296,6 @@
     <t>R21</t>
   </si>
   <si>
-    <t>CRCW0805220KFKEA</t>
-  </si>
-  <si>
-    <t>71-CRCW0805220KFKEA</t>
-  </si>
-  <si>
     <t>SW1, SW2</t>
   </si>
   <si>
@@ -410,7 +371,67 @@
     <t>4mm Banana Socket B</t>
   </si>
   <si>
-    <t>845-973582100</t>
+    <t>LIB_24.243.1:24.243.1</t>
+  </si>
+  <si>
+    <t>Multicomp 24.243.1</t>
+  </si>
+  <si>
+    <t>LIB_24.243.1:24.243.2</t>
+  </si>
+  <si>
+    <t>Multicomp 24.243.2</t>
+  </si>
+  <si>
+    <t>Molex 39-30-1240</t>
+  </si>
+  <si>
+    <t>39-30-1240</t>
+  </si>
+  <si>
+    <t>Molex 172448-0008</t>
+  </si>
+  <si>
+    <t>172448-0008</t>
+  </si>
+  <si>
+    <t>ADDR: 0x3C/0x3D</t>
+  </si>
+  <si>
+    <t>J12, J13, J14, J15, J16, J17, J21</t>
+  </si>
+  <si>
+    <t>R16, R17</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>538-39-30-1240</t>
+  </si>
+  <si>
+    <t>538-172448-0008</t>
+  </si>
+  <si>
+    <t>Mouser Bom Copy + Pase</t>
+  </si>
+  <si>
+    <t>Extra</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>CRCW0805220RFKEAC</t>
+  </si>
+  <si>
+    <t>71-CRCW0805220RFKEAC</t>
+  </si>
+  <si>
+    <t>SKHHBWA010</t>
+  </si>
+  <si>
+    <t>688-SKHHBW</t>
   </si>
 </sst>
 </file>
@@ -894,9 +915,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1272,13 +1294,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7BD461-B7D6-4F3C-850A-669DBD31CA72}">
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="20" max="20" width="37.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="6.85546875" customWidth="1"/>
+    <col min="9" max="9" width="7.5703125" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" customWidth="1"/>
+    <col min="12" max="12" width="5.5703125" customWidth="1"/>
+    <col min="13" max="13" width="5.28515625" customWidth="1"/>
+    <col min="14" max="14" width="4.28515625" customWidth="1"/>
+    <col min="18" max="18" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1286,15 +1316,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1">
-        <v>46125.002881944441</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>46131.071944444448</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1302,7 +1332,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1310,55 +1340,64 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="O9" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1380,29 +1419,25 @@
       <c r="G10" t="s">
         <v>24</v>
       </c>
+      <c r="J10" t="s">
+        <v>25</v>
+      </c>
       <c r="K10" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" t="s">
         <v>26</v>
       </c>
       <c r="O10">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P10">
         <f>B10+O10</f>
-        <v>27</v>
-      </c>
-      <c r="Q10" t="str">
-        <f>L10</f>
-        <v>581-08055C104J</v>
-      </c>
-      <c r="T10" t="str">
-        <f>IF(ISBLANK(O10), "", Q10&amp;"|"&amp;P10)</f>
-        <v>581-08055C104J|27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="R10" t="str">
+        <f>IF(ISBLANK(K10), "",K10&amp; "|"&amp;P10)</f>
+        <v>581-08055C104J|30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1424,29 +1459,25 @@
       <c r="G11" t="s">
         <v>24</v>
       </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
       <c r="K11" t="s">
-        <v>29</v>
-      </c>
-      <c r="L11" t="s">
         <v>30</v>
       </c>
       <c r="O11">
         <v>8</v>
       </c>
       <c r="P11">
-        <f t="shared" ref="P11:P32" si="0">B11+O11</f>
+        <f t="shared" ref="P11:P33" si="0">B11+O11</f>
         <v>10</v>
       </c>
-      <c r="Q11" t="str">
-        <f t="shared" ref="Q11:Q32" si="1">L11</f>
-        <v>581-KGM21AR71C105JU</v>
-      </c>
-      <c r="T11" t="str">
-        <f t="shared" ref="T11:T32" si="2">IF(ISBLANK(O11), "", Q11&amp;"|"&amp;P11)</f>
+      <c r="R11" t="str">
+        <f t="shared" ref="R11:R33" si="1">IF(ISBLANK(K11), "",K11&amp; "|"&amp;P11)</f>
         <v>581-KGM21AR71C105JU|10</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1468,12 +1499,16 @@
       <c r="G12" t="s">
         <v>24</v>
       </c>
-      <c r="T12" t="str">
-        <f t="shared" si="2"/>
+      <c r="P12">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="R12" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1481,43 +1516,33 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="E13" t="s">
         <v>35</v>
       </c>
       <c r="F13" t="s">
-        <v>36</v>
+        <v>112</v>
       </c>
       <c r="G13" t="s">
         <v>24</v>
       </c>
-      <c r="K13">
-        <v>973582101</v>
-      </c>
-      <c r="L13" t="s">
-        <v>37</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
+      <c r="J13" t="s">
+        <v>113</v>
       </c>
       <c r="P13">
-        <f t="shared" ref="P13" si="3">B13+O13</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="Q13" t="str">
-        <f t="shared" ref="Q13" si="4">L13</f>
-        <v>845-973582101</v>
-      </c>
-      <c r="T13" t="str">
-        <f t="shared" si="2"/>
-        <v>845-973582101|5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="R13" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1525,43 +1550,33 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="E14" t="s">
         <v>35</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>114</v>
       </c>
       <c r="G14" t="s">
         <v>24</v>
       </c>
-      <c r="K14">
-        <v>973582100</v>
-      </c>
-      <c r="L14" t="s">
-        <v>125</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
+      <c r="J14" t="s">
+        <v>115</v>
       </c>
       <c r="P14">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="R14" t="str">
         <f t="shared" si="1"/>
-        <v>845-973582100</v>
-      </c>
-      <c r="T14" t="str">
-        <f t="shared" si="2"/>
-        <v>845-973582100|3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6</v>
       </c>
@@ -1569,43 +1584,39 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" t="s">
         <v>38</v>
       </c>
-      <c r="D15" t="s">
+      <c r="G15" t="s">
         <v>39</v>
       </c>
-      <c r="E15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F15" t="s">
-        <v>41</v>
-      </c>
-      <c r="G15" t="s">
-        <v>42</v>
+      <c r="J15" t="s">
+        <v>117</v>
       </c>
       <c r="K15" t="s">
-        <v>43</v>
-      </c>
-      <c r="L15" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="Q15" t="str">
+        <v>2</v>
+      </c>
+      <c r="R15" t="str">
         <f t="shared" si="1"/>
-        <v>538-39-30-1241</v>
-      </c>
-      <c r="T15" t="str">
-        <f t="shared" si="2"/>
-        <v>538-39-30-1241|1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+        <v>538-39-30-1240|2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>7</v>
       </c>
@@ -1613,43 +1624,39 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>118</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G16" t="s">
         <v>24</v>
       </c>
+      <c r="J16" t="s">
+        <v>119</v>
+      </c>
       <c r="K16" t="s">
-        <v>49</v>
-      </c>
-      <c r="L16" t="s">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P16">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="Q16" t="str">
+        <v>2</v>
+      </c>
+      <c r="R16" t="str">
         <f t="shared" si="1"/>
-        <v>538-46991-1008</v>
-      </c>
-      <c r="T16" t="str">
-        <f t="shared" si="2"/>
-        <v>538-46991-1008|1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+        <v>538-172448-0008|2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>8</v>
       </c>
@@ -1657,53 +1664,61 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="F17" t="s">
-        <v>53</v>
-      </c>
-      <c r="J17" t="s">
-        <v>54</v>
-      </c>
-      <c r="T17" t="str">
-        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+      <c r="I17" t="s">
+        <v>120</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="R17" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E18" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F18" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G18" t="s">
         <v>24</v>
       </c>
-      <c r="T18" t="str">
-        <f t="shared" si="2"/>
+      <c r="P18">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="R18" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>10</v>
       </c>
@@ -1711,26 +1726,30 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F19" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G19" t="s">
         <v>24</v>
       </c>
-      <c r="T19" t="str">
-        <f t="shared" si="2"/>
+      <c r="P19">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="R19" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>11</v>
       </c>
@@ -1738,26 +1757,30 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E20" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F20" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="G20" t="s">
         <v>24</v>
       </c>
-      <c r="T20" t="str">
-        <f t="shared" si="2"/>
+      <c r="P20">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="R20" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>12</v>
       </c>
@@ -1765,26 +1788,30 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E21" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G21" t="s">
         <v>24</v>
       </c>
-      <c r="T21" t="str">
-        <f t="shared" si="2"/>
+      <c r="P21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="R21" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>13</v>
       </c>
@@ -1792,25 +1819,25 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G22" t="s">
         <v>24</v>
       </c>
+      <c r="J22" t="s">
+        <v>62</v>
+      </c>
       <c r="K22" t="s">
-        <v>72</v>
-      </c>
-      <c r="L22" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="O22">
         <v>4</v>
@@ -1819,16 +1846,12 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="Q22" t="str">
+      <c r="R22" t="str">
         <f t="shared" si="1"/>
-        <v>863-50C02CH-TL-E</v>
-      </c>
-      <c r="T22" t="str">
-        <f t="shared" si="2"/>
         <v>863-50C02CH-TL-E|5</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>14</v>
       </c>
@@ -1836,25 +1859,25 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="D23">
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F23" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G23" t="s">
         <v>24</v>
       </c>
+      <c r="J23" t="s">
+        <v>69</v>
+      </c>
       <c r="K23" t="s">
-        <v>79</v>
-      </c>
-      <c r="L23" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O23">
         <v>10</v>
@@ -1863,16 +1886,12 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="Q23" t="str">
+      <c r="R23" t="str">
         <f t="shared" si="1"/>
-        <v>71-CRCW0805-10-E3</v>
-      </c>
-      <c r="T23" t="str">
-        <f t="shared" si="2"/>
         <v>71-CRCW0805-10-E3|20</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>15</v>
       </c>
@@ -1880,87 +1899,82 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="D24">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="E24" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="G24" t="s">
         <v>24</v>
       </c>
+      <c r="J24" t="s">
+        <v>73</v>
+      </c>
       <c r="K24" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P24">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="Q24" t="str">
+        <v>15</v>
+      </c>
+      <c r="R24" t="str">
         <f t="shared" si="1"/>
-        <v>504-MSMA2512R0050FEN</v>
-      </c>
-      <c r="T24" t="str">
-        <f t="shared" si="2"/>
-        <v>504-MSMA2512R0050FEN|5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+        <v>504-MSMA2512R0050FEN|15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>16</v>
       </c>
       <c r="B25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="D25" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="E25" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F25" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G25" t="s">
         <v>24</v>
       </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25" t="s">
+        <v>76</v>
+      </c>
       <c r="K25" t="s">
-        <v>87</v>
-      </c>
-      <c r="L25" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="O25">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P25">
         <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="Q25" t="str">
+        <v>10</v>
+      </c>
+      <c r="R25" t="str">
         <f t="shared" si="1"/>
-        <v>71-CRCW0805-1.65K-E3</v>
-      </c>
-      <c r="T25" t="str">
-        <f t="shared" si="2"/>
-        <v>71-CRCW0805-1.65K-E3|13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+        <v>71-CRCW0805-1.65K-E3|10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>17</v>
       </c>
@@ -1968,25 +1982,25 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E26" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F26" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G26" t="s">
         <v>24</v>
       </c>
+      <c r="J26" t="s">
+        <v>80</v>
+      </c>
       <c r="K26" t="s">
-        <v>91</v>
-      </c>
-      <c r="L26" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="O26">
         <v>10</v>
@@ -1995,16 +2009,12 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="Q26" t="str">
+      <c r="R26" t="str">
         <f t="shared" si="1"/>
-        <v>71-CRCW0805-1.0K-E3</v>
-      </c>
-      <c r="T26" t="str">
-        <f t="shared" si="2"/>
         <v>71-CRCW0805-1.0K-E3|11</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>18</v>
       </c>
@@ -2012,25 +2022,25 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="D27" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E27" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F27" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
+      <c r="J27" t="s">
+        <v>76</v>
+      </c>
       <c r="K27" t="s">
-        <v>95</v>
-      </c>
-      <c r="L27" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="O27">
         <v>10</v>
@@ -2039,16 +2049,12 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="Q27" t="str">
+      <c r="R27" t="str">
         <f t="shared" si="1"/>
-        <v>71-CRCW0805-3.3K-E3</v>
-      </c>
-      <c r="T27" t="str">
-        <f t="shared" si="2"/>
-        <v>71-CRCW0805-3.3K-E3|11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+        <v>71-CRCW0805-1.65K-E3|11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>19</v>
       </c>
@@ -2056,25 +2062,25 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
-      </c>
-      <c r="D28">
-        <v>220</v>
+        <v>82</v>
+      </c>
+      <c r="D28" t="s">
+        <v>83</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G28" t="s">
         <v>24</v>
       </c>
+      <c r="J28" t="s">
+        <v>84</v>
+      </c>
       <c r="K28" t="s">
-        <v>98</v>
-      </c>
-      <c r="L28" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="O28">
         <v>10</v>
@@ -2083,155 +2089,201 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="Q28" t="str">
+      <c r="R28" t="str">
         <f t="shared" si="1"/>
-        <v>71-CRCW0805220KFKEA</v>
-      </c>
-      <c r="T28" t="str">
-        <f t="shared" si="2"/>
-        <v>71-CRCW0805220KFKEA|11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+        <v>71-CRCW0805-3.3K-E3|11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>20</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>100</v>
-      </c>
-      <c r="D29" t="s">
-        <v>101</v>
+        <v>86</v>
+      </c>
+      <c r="D29">
+        <v>220</v>
       </c>
       <c r="E29" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="F29" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="G29" t="s">
         <v>24</v>
       </c>
-      <c r="T29" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="J29" t="s">
+        <v>129</v>
+      </c>
+      <c r="K29" t="s">
+        <v>130</v>
+      </c>
+      <c r="O29">
+        <v>10</v>
+      </c>
+      <c r="P29">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="R29" t="str">
+        <f t="shared" si="1"/>
+        <v>71-CRCW0805220RFKEAC|11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>21</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="D30" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="F30" t="s">
-        <v>107</v>
-      </c>
-      <c r="T30" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="G30" t="s">
+        <v>24</v>
+      </c>
+      <c r="J30" t="s">
+        <v>131</v>
+      </c>
+      <c r="K30" t="s">
+        <v>132</v>
+      </c>
+      <c r="O30">
+        <v>8</v>
+      </c>
+      <c r="P30">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R30" t="str">
+        <f t="shared" si="1"/>
+        <v>688-SKHHBW|10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>22</v>
       </c>
       <c r="B31">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="E31" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="F31" t="s">
-        <v>111</v>
-      </c>
-      <c r="G31" t="s">
-        <v>112</v>
-      </c>
-      <c r="K31" t="s">
-        <v>109</v>
-      </c>
-      <c r="L31" t="s">
-        <v>113</v>
-      </c>
-      <c r="O31">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="P31">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="Q31" t="str">
+        <v>1</v>
+      </c>
+      <c r="R31" t="str">
         <f t="shared" si="1"/>
-        <v>595-INA219BIDR</v>
-      </c>
-      <c r="T31" t="str">
-        <f t="shared" si="2"/>
-        <v>595-INA219BIDR|10</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>23</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D32" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="E32" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="F32" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="G32" t="s">
-        <v>118</v>
+        <v>99</v>
+      </c>
+      <c r="J32" t="s">
+        <v>96</v>
       </c>
       <c r="K32" t="s">
-        <v>119</v>
-      </c>
-      <c r="L32" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="O32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P32">
         <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R32" t="str">
+        <f t="shared" si="1"/>
+        <v>595-INA219BIDR|10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>24</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" t="s">
+        <v>102</v>
+      </c>
+      <c r="E33" t="s">
+        <v>103</v>
+      </c>
+      <c r="F33" t="s">
+        <v>104</v>
+      </c>
+      <c r="G33" t="s">
+        <v>105</v>
+      </c>
+      <c r="J33" t="s">
+        <v>106</v>
+      </c>
+      <c r="K33" t="s">
+        <v>107</v>
+      </c>
+      <c r="O33">
+        <v>4</v>
+      </c>
+      <c r="P33">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="Q32" t="str">
+      <c r="R33" t="str">
         <f t="shared" si="1"/>
-        <v>595-TLV75733PDBVR</v>
-      </c>
-      <c r="T32" t="str">
-        <f t="shared" si="2"/>
         <v>595-TLV75733PDBVR|5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>